<commit_message>
Honduras area drivers: production since 1960 with year-over-year change
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GCSUFXh2mYdWNgg7VCeE1G
</commit_message>
<xml_diff>
--- a/research/honduras/excel/Honduras_area_drivers.xlsx
+++ b/research/honduras/excel/Honduras_area_drivers.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Margin" sheetId="4" r:id="rId4"/>
     <sheet name="Rust_2012" sheetId="5" r:id="rId5"/>
     <sheet name="USDA_quotes" sheetId="6" r:id="rId6"/>
+    <sheet name="Production_1960_2026" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -225,35 +226,42 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Production_1960_2026 : la production USDA du Honduras depuis 1960/61, avec la variation d'une année sur l'autre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">À SAVOIR AVANT D'INTERPRÉTER</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">Les nombres d'arbres de l'USDA sont des estimations : 1 049 millions chaque année de 2006 à 2010, puis une densité fixe d'environ 4 250 arbres/ha jusqu'en 2017, et 6 400/ha depuis 2023. Depuis 2020, les deux tiers de la hausse des arbres viennent de cette densité, pas de nouvelles surfaces.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">La FAO marque la surface de café du Honduras comme imputée depuis 2013 et le prix producteur comme estimé : non utilisés.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La FAO marque la surface de café du Honduras comme imputée depuis 2013 et le prix producteur comme estimé : non utilisés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Le registre de l'IHCAFE (surface récoltée des fermes inscrites) baisse de 315 700 ha (2022/23) à 280 100 (2023/24) puis 285 600 ha (2024/25), alors que l'USDA l'augmente : la hausse récente de la surface est incertaine.</t>
         </is>
@@ -5906,4 +5914,1389 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="13.2"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marketing year (Oct N – Sep N+1)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Year N</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Production (1000 bags 60 kg)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Change on the year before</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bean exports (1000 bags)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1960/61</t>
+        </is>
+      </c>
+      <c r="B2" s="2">
+        <v>1960</v>
+      </c>
+      <c r="C2" s="3">
+        <v>291.0</v>
+      </c>
+      <c r="E2" s="3">
+        <v>225.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1961/62</t>
+        </is>
+      </c>
+      <c r="B3" s="2">
+        <v>1961</v>
+      </c>
+      <c r="C3" s="3">
+        <v>315.0</v>
+      </c>
+      <c r="D3" s="9">
+        <f>IF(C2=0,"",C3/C2-1)</f>
+        <v>0.08247422680412364</v>
+      </c>
+      <c r="E3" s="3">
+        <v>247.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1962/63</t>
+        </is>
+      </c>
+      <c r="B4" s="2">
+        <v>1962</v>
+      </c>
+      <c r="C4" s="3">
+        <v>405.0</v>
+      </c>
+      <c r="D4" s="9">
+        <f>IF(C3=0,"",C4/C3-1)</f>
+        <v>0.2857142857142858</v>
+      </c>
+      <c r="E4" s="3">
+        <v>334.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1963/64</t>
+        </is>
+      </c>
+      <c r="B5" s="2">
+        <v>1963</v>
+      </c>
+      <c r="C5" s="3">
+        <v>390.0</v>
+      </c>
+      <c r="D5" s="9">
+        <f>IF(C4=0,"",C5/C4-1)</f>
+        <v>-0.03703703703703709</v>
+      </c>
+      <c r="E5" s="3">
+        <v>317.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1964/65</t>
+        </is>
+      </c>
+      <c r="B6" s="2">
+        <v>1964</v>
+      </c>
+      <c r="C6" s="3">
+        <v>479.0</v>
+      </c>
+      <c r="D6" s="9">
+        <f>IF(C5=0,"",C6/C5-1)</f>
+        <v>0.22820512820512828</v>
+      </c>
+      <c r="E6" s="3">
+        <v>404.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1965/66</t>
+        </is>
+      </c>
+      <c r="B7" s="2">
+        <v>1965</v>
+      </c>
+      <c r="C7" s="3">
+        <v>461.0</v>
+      </c>
+      <c r="D7" s="9">
+        <f>IF(C6=0,"",C7/C6-1)</f>
+        <v>-0.0375782881002088</v>
+      </c>
+      <c r="E7" s="3">
+        <v>383.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1966/67</t>
+        </is>
+      </c>
+      <c r="B8" s="2">
+        <v>1966</v>
+      </c>
+      <c r="C8" s="3">
+        <v>431.0</v>
+      </c>
+      <c r="D8" s="9">
+        <f>IF(C7=0,"",C8/C7-1)</f>
+        <v>-0.06507592190889366</v>
+      </c>
+      <c r="E8" s="3">
+        <v>351.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1967/68</t>
+        </is>
+      </c>
+      <c r="B9" s="2">
+        <v>1967</v>
+      </c>
+      <c r="C9" s="3">
+        <v>495.0</v>
+      </c>
+      <c r="D9" s="9">
+        <f>IF(C8=0,"",C9/C8-1)</f>
+        <v>0.14849187935034802</v>
+      </c>
+      <c r="E9" s="3">
+        <v>413.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1968/69</t>
+        </is>
+      </c>
+      <c r="B10" s="2">
+        <v>1968</v>
+      </c>
+      <c r="C10" s="3">
+        <v>514.0</v>
+      </c>
+      <c r="D10" s="9">
+        <f>IF(C9=0,"",C10/C9-1)</f>
+        <v>0.03838383838383841</v>
+      </c>
+      <c r="E10" s="3">
+        <v>364.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1969/70</t>
+        </is>
+      </c>
+      <c r="B11" s="2">
+        <v>1969</v>
+      </c>
+      <c r="C11" s="3">
+        <v>443.0</v>
+      </c>
+      <c r="D11" s="9">
+        <f>IF(C10=0,"",C11/C10-1)</f>
+        <v>-0.1381322957198443</v>
+      </c>
+      <c r="E11" s="3">
+        <v>470.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1970/71</t>
+        </is>
+      </c>
+      <c r="B12" s="2">
+        <v>1970</v>
+      </c>
+      <c r="C12" s="3">
+        <v>545.0</v>
+      </c>
+      <c r="D12" s="9">
+        <f>IF(C11=0,"",C12/C11-1)</f>
+        <v>0.23024830699774257</v>
+      </c>
+      <c r="E12" s="3">
+        <v>379.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1971/72</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <v>1971</v>
+      </c>
+      <c r="C13" s="3">
+        <v>586.0</v>
+      </c>
+      <c r="D13" s="9">
+        <f>IF(C12=0,"",C13/C12-1)</f>
+        <v>0.07522935779816509</v>
+      </c>
+      <c r="E13" s="3">
+        <v>560.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1972/73</t>
+        </is>
+      </c>
+      <c r="B14" s="2">
+        <v>1972</v>
+      </c>
+      <c r="C14" s="3">
+        <v>759.0</v>
+      </c>
+      <c r="D14" s="9">
+        <f>IF(C13=0,"",C14/C13-1)</f>
+        <v>0.29522184300341303</v>
+      </c>
+      <c r="E14" s="3">
+        <v>686.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1973/74</t>
+        </is>
+      </c>
+      <c r="B15" s="2">
+        <v>1973</v>
+      </c>
+      <c r="C15" s="3">
+        <v>689.0</v>
+      </c>
+      <c r="D15" s="9">
+        <f>IF(C14=0,"",C15/C14-1)</f>
+        <v>-0.09222661396574439</v>
+      </c>
+      <c r="E15" s="3">
+        <v>477.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1974/75</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>1974</v>
+      </c>
+      <c r="C16" s="3">
+        <v>983.0</v>
+      </c>
+      <c r="D16" s="9">
+        <f>IF(C15=0,"",C16/C15-1)</f>
+        <v>0.4267053701015966</v>
+      </c>
+      <c r="E16" s="3">
+        <v>857.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1975/76</t>
+        </is>
+      </c>
+      <c r="B17" s="2">
+        <v>1975</v>
+      </c>
+      <c r="C17" s="3">
+        <v>847.0</v>
+      </c>
+      <c r="D17" s="9">
+        <f>IF(C16=0,"",C17/C16-1)</f>
+        <v>-0.13835198372329605</v>
+      </c>
+      <c r="E17" s="3">
+        <v>832.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1976/77</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <v>1976</v>
+      </c>
+      <c r="C18" s="3">
+        <v>691.0</v>
+      </c>
+      <c r="D18" s="9">
+        <f>IF(C17=0,"",C18/C17-1)</f>
+        <v>-0.18417945690672965</v>
+      </c>
+      <c r="E18" s="3">
+        <v>640.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1977/78</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <v>1977</v>
+      </c>
+      <c r="C19" s="3">
+        <v>1036.0</v>
+      </c>
+      <c r="D19" s="9">
+        <f>IF(C18=0,"",C19/C18-1)</f>
+        <v>0.4992764109985528</v>
+      </c>
+      <c r="E19" s="3">
+        <v>939.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1978/79</t>
+        </is>
+      </c>
+      <c r="B20" s="2">
+        <v>1978</v>
+      </c>
+      <c r="C20" s="3">
+        <v>1132.0</v>
+      </c>
+      <c r="D20" s="9">
+        <f>IF(C19=0,"",C20/C19-1)</f>
+        <v>0.0926640926640927</v>
+      </c>
+      <c r="E20" s="3">
+        <v>1051.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1979/80</t>
+        </is>
+      </c>
+      <c r="B21" s="2">
+        <v>1979</v>
+      </c>
+      <c r="C21" s="3">
+        <v>1137.0</v>
+      </c>
+      <c r="D21" s="9">
+        <f>IF(C20=0,"",C21/C20-1)</f>
+        <v>0.004416961130742081</v>
+      </c>
+      <c r="E21" s="3">
+        <v>980.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1980/81</t>
+        </is>
+      </c>
+      <c r="B22" s="2">
+        <v>1980</v>
+      </c>
+      <c r="C22" s="3">
+        <v>1265.0</v>
+      </c>
+      <c r="D22" s="9">
+        <f>IF(C21=0,"",C22/C21-1)</f>
+        <v>0.11257695690413372</v>
+      </c>
+      <c r="E22" s="3">
+        <v>1030.0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1981/82</t>
+        </is>
+      </c>
+      <c r="B23" s="2">
+        <v>1981</v>
+      </c>
+      <c r="C23" s="3">
+        <v>1200.0</v>
+      </c>
+      <c r="D23" s="9">
+        <f>IF(C22=0,"",C23/C22-1)</f>
+        <v>-0.0513833992094862</v>
+      </c>
+      <c r="E23" s="3">
+        <v>911.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1982/83</t>
+        </is>
+      </c>
+      <c r="B24" s="2">
+        <v>1982</v>
+      </c>
+      <c r="C24" s="3">
+        <v>1500.0</v>
+      </c>
+      <c r="D24" s="9">
+        <f>IF(C23=0,"",C24/C23-1)</f>
+        <v>0.25</v>
+      </c>
+      <c r="E24" s="3">
+        <v>1146.0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1983/84</t>
+        </is>
+      </c>
+      <c r="B25" s="2">
+        <v>1983</v>
+      </c>
+      <c r="C25" s="3">
+        <v>1310.0</v>
+      </c>
+      <c r="D25" s="9">
+        <f>IF(C24=0,"",C25/C24-1)</f>
+        <v>-0.1266666666666667</v>
+      </c>
+      <c r="E25" s="3">
+        <v>1050.0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1984/85</t>
+        </is>
+      </c>
+      <c r="B26" s="2">
+        <v>1984</v>
+      </c>
+      <c r="C26" s="3">
+        <v>1400.0</v>
+      </c>
+      <c r="D26" s="9">
+        <f>IF(C25=0,"",C26/C25-1)</f>
+        <v>0.06870229007633588</v>
+      </c>
+      <c r="E26" s="3">
+        <v>1281.0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1985/86</t>
+        </is>
+      </c>
+      <c r="B27" s="2">
+        <v>1985</v>
+      </c>
+      <c r="C27" s="3">
+        <v>1062.0</v>
+      </c>
+      <c r="D27" s="9">
+        <f>IF(C26=0,"",C27/C26-1)</f>
+        <v>-0.24142857142857144</v>
+      </c>
+      <c r="E27" s="3">
+        <v>1481.0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1986/87</t>
+        </is>
+      </c>
+      <c r="B28" s="2">
+        <v>1986</v>
+      </c>
+      <c r="C28" s="3">
+        <v>1535.0</v>
+      </c>
+      <c r="D28" s="9">
+        <f>IF(C27=0,"",C28/C27-1)</f>
+        <v>0.4453860640301319</v>
+      </c>
+      <c r="E28" s="3">
+        <v>1398.0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1987/88</t>
+        </is>
+      </c>
+      <c r="B29" s="2">
+        <v>1987</v>
+      </c>
+      <c r="C29" s="3">
+        <v>1553.0</v>
+      </c>
+      <c r="D29" s="9">
+        <f>IF(C28=0,"",C29/C28-1)</f>
+        <v>0.011726384364820763</v>
+      </c>
+      <c r="E29" s="3">
+        <v>1224.0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1988/89</t>
+        </is>
+      </c>
+      <c r="B30" s="2">
+        <v>1988</v>
+      </c>
+      <c r="C30" s="3">
+        <v>1635.0</v>
+      </c>
+      <c r="D30" s="9">
+        <f>IF(C29=0,"",C30/C29-1)</f>
+        <v>0.05280103026400518</v>
+      </c>
+      <c r="E30" s="3">
+        <v>1464.0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1989/90</t>
+        </is>
+      </c>
+      <c r="B31" s="2">
+        <v>1989</v>
+      </c>
+      <c r="C31" s="3">
+        <v>1928.0</v>
+      </c>
+      <c r="D31" s="9">
+        <f>IF(C30=0,"",C31/C30-1)</f>
+        <v>0.17920489296636077</v>
+      </c>
+      <c r="E31" s="3">
+        <v>1810.0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1990/91</t>
+        </is>
+      </c>
+      <c r="B32" s="2">
+        <v>1990</v>
+      </c>
+      <c r="C32" s="3">
+        <v>1685.0</v>
+      </c>
+      <c r="D32" s="9">
+        <f>IF(C31=0,"",C32/C31-1)</f>
+        <v>-0.12603734439834025</v>
+      </c>
+      <c r="E32" s="3">
+        <v>1490.0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1991/92</t>
+        </is>
+      </c>
+      <c r="B33" s="2">
+        <v>1991</v>
+      </c>
+      <c r="C33" s="3">
+        <v>2255.0</v>
+      </c>
+      <c r="D33" s="9">
+        <f>IF(C32=0,"",C33/C32-1)</f>
+        <v>0.33827893175074175</v>
+      </c>
+      <c r="E33" s="3">
+        <v>1800.0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1992/93</t>
+        </is>
+      </c>
+      <c r="B34" s="2">
+        <v>1992</v>
+      </c>
+      <c r="C34" s="3">
+        <v>1981.0</v>
+      </c>
+      <c r="D34" s="9">
+        <f>IF(C33=0,"",C34/C33-1)</f>
+        <v>-0.12150776053215073</v>
+      </c>
+      <c r="E34" s="3">
+        <v>2042.0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1993/94</t>
+        </is>
+      </c>
+      <c r="B35" s="2">
+        <v>1993</v>
+      </c>
+      <c r="C35" s="3">
+        <v>2060.0</v>
+      </c>
+      <c r="D35" s="9">
+        <f>IF(C34=0,"",C35/C34-1)</f>
+        <v>0.03987884906612815</v>
+      </c>
+      <c r="E35" s="3">
+        <v>1815.0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1994/95</t>
+        </is>
+      </c>
+      <c r="B36" s="2">
+        <v>1994</v>
+      </c>
+      <c r="C36" s="3">
+        <v>2295.0</v>
+      </c>
+      <c r="D36" s="9">
+        <f>IF(C35=0,"",C36/C35-1)</f>
+        <v>0.11407766990291268</v>
+      </c>
+      <c r="E36" s="3">
+        <v>1753.0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1995/96</t>
+        </is>
+      </c>
+      <c r="B37" s="2">
+        <v>1995</v>
+      </c>
+      <c r="C37" s="3">
+        <v>2254.0</v>
+      </c>
+      <c r="D37" s="9">
+        <f>IF(C36=0,"",C37/C36-1)</f>
+        <v>-0.017864923747276662</v>
+      </c>
+      <c r="E37" s="3">
+        <v>2279.0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1996/97</t>
+        </is>
+      </c>
+      <c r="B38" s="2">
+        <v>1996</v>
+      </c>
+      <c r="C38" s="3">
+        <v>2279.0</v>
+      </c>
+      <c r="D38" s="9">
+        <f>IF(C37=0,"",C38/C37-1)</f>
+        <v>0.011091393078970668</v>
+      </c>
+      <c r="E38" s="3">
+        <v>2025.0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1997/98</t>
+        </is>
+      </c>
+      <c r="B39" s="2">
+        <v>1997</v>
+      </c>
+      <c r="C39" s="3">
+        <v>2905.0</v>
+      </c>
+      <c r="D39" s="9">
+        <f>IF(C38=0,"",C39/C38-1)</f>
+        <v>0.274681878016674</v>
+      </c>
+      <c r="E39" s="3">
+        <v>2554.0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1998/99</t>
+        </is>
+      </c>
+      <c r="B40" s="2">
+        <v>1998</v>
+      </c>
+      <c r="C40" s="3">
+        <v>2494.0</v>
+      </c>
+      <c r="D40" s="9">
+        <f>IF(C39=0,"",C40/C39-1)</f>
+        <v>-0.14148020654044746</v>
+      </c>
+      <c r="E40" s="3">
+        <v>2255.0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1999/00</t>
+        </is>
+      </c>
+      <c r="B41" s="2">
+        <v>1999</v>
+      </c>
+      <c r="C41" s="3">
+        <v>3067.0</v>
+      </c>
+      <c r="D41" s="9">
+        <f>IF(C40=0,"",C41/C40-1)</f>
+        <v>0.22975140336808342</v>
+      </c>
+      <c r="E41" s="3">
+        <v>2825.0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2000/01</t>
+        </is>
+      </c>
+      <c r="B42" s="2">
+        <v>2000</v>
+      </c>
+      <c r="C42" s="3">
+        <v>2821.0</v>
+      </c>
+      <c r="D42" s="9">
+        <f>IF(C41=0,"",C42/C41-1)</f>
+        <v>-0.0802086729703293</v>
+      </c>
+      <c r="E42" s="3">
+        <v>2470.0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2001/02</t>
+        </is>
+      </c>
+      <c r="B43" s="2">
+        <v>2001</v>
+      </c>
+      <c r="C43" s="3">
+        <v>3098.0</v>
+      </c>
+      <c r="D43" s="9">
+        <f>IF(C42=0,"",C43/C42-1)</f>
+        <v>0.09819213045019493</v>
+      </c>
+      <c r="E43" s="3">
+        <v>2617.0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2002/03</t>
+        </is>
+      </c>
+      <c r="B44" s="2">
+        <v>2002</v>
+      </c>
+      <c r="C44" s="3">
+        <v>2496.0</v>
+      </c>
+      <c r="D44" s="9">
+        <f>IF(C43=0,"",C44/C43-1)</f>
+        <v>-0.19431891542930924</v>
+      </c>
+      <c r="E44" s="3">
+        <v>2438.0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2003/04</t>
+        </is>
+      </c>
+      <c r="B45" s="2">
+        <v>2003</v>
+      </c>
+      <c r="C45" s="3">
+        <v>2968.0</v>
+      </c>
+      <c r="D45" s="9">
+        <f>IF(C44=0,"",C45/C44-1)</f>
+        <v>0.1891025641025641</v>
+      </c>
+      <c r="E45" s="3">
+        <v>2794.0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2004/05</t>
+        </is>
+      </c>
+      <c r="B46" s="2">
+        <v>2004</v>
+      </c>
+      <c r="C46" s="3">
+        <v>2575.0</v>
+      </c>
+      <c r="D46" s="9">
+        <f>IF(C45=0,"",C46/C45-1)</f>
+        <v>-0.13241239892183287</v>
+      </c>
+      <c r="E46" s="3">
+        <v>2450.0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2005/06</t>
+        </is>
+      </c>
+      <c r="B47" s="2">
+        <v>2005</v>
+      </c>
+      <c r="C47" s="3">
+        <v>3204.0</v>
+      </c>
+      <c r="D47" s="9">
+        <f>IF(C46=0,"",C47/C46-1)</f>
+        <v>0.24427184466019414</v>
+      </c>
+      <c r="E47" s="3">
+        <v>2850.0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2006/07</t>
+        </is>
+      </c>
+      <c r="B48" s="2">
+        <v>2006</v>
+      </c>
+      <c r="C48" s="3">
+        <v>3460.0</v>
+      </c>
+      <c r="D48" s="9">
+        <f>IF(C47=0,"",C48/C47-1)</f>
+        <v>0.07990012484394504</v>
+      </c>
+      <c r="E48" s="3">
+        <v>3370.0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2007/08</t>
+        </is>
+      </c>
+      <c r="B49" s="2">
+        <v>2007</v>
+      </c>
+      <c r="C49" s="3">
+        <v>3642.0</v>
+      </c>
+      <c r="D49" s="9">
+        <f>IF(C48=0,"",C49/C48-1)</f>
+        <v>0.05260115606936422</v>
+      </c>
+      <c r="E49" s="3">
+        <v>3440.0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2008/09</t>
+        </is>
+      </c>
+      <c r="B50" s="2">
+        <v>2008</v>
+      </c>
+      <c r="C50" s="3">
+        <v>3225.0</v>
+      </c>
+      <c r="D50" s="9">
+        <f>IF(C49=0,"",C50/C49-1)</f>
+        <v>-0.11449752883031306</v>
+      </c>
+      <c r="E50" s="3">
+        <v>3050.0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2009/10</t>
+        </is>
+      </c>
+      <c r="B51" s="2">
+        <v>2009</v>
+      </c>
+      <c r="C51" s="3">
+        <v>3550.0</v>
+      </c>
+      <c r="D51" s="9">
+        <f>IF(C50=0,"",C51/C50-1)</f>
+        <v>0.10077519379844957</v>
+      </c>
+      <c r="E51" s="3">
+        <v>3200.0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2010/11</t>
+        </is>
+      </c>
+      <c r="B52" s="2">
+        <v>2010</v>
+      </c>
+      <c r="C52" s="3">
+        <v>3975.0</v>
+      </c>
+      <c r="D52" s="9">
+        <f>IF(C51=0,"",C52/C51-1)</f>
+        <v>0.11971830985915499</v>
+      </c>
+      <c r="E52" s="3">
+        <v>3900.0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2011/12</t>
+        </is>
+      </c>
+      <c r="B53" s="2">
+        <v>2011</v>
+      </c>
+      <c r="C53" s="3">
+        <v>5600.0</v>
+      </c>
+      <c r="D53" s="9">
+        <f>IF(C52=0,"",C53/C52-1)</f>
+        <v>0.4088050314465408</v>
+      </c>
+      <c r="E53" s="3">
+        <v>5290.0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2012/13</t>
+        </is>
+      </c>
+      <c r="B54" s="2">
+        <v>2012</v>
+      </c>
+      <c r="C54" s="3">
+        <v>4725.0</v>
+      </c>
+      <c r="D54" s="9">
+        <f>IF(C53=0,"",C54/C53-1)</f>
+        <v>-0.15625</v>
+      </c>
+      <c r="E54" s="3">
+        <v>4480.0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2013/14</t>
+        </is>
+      </c>
+      <c r="B55" s="2">
+        <v>2013</v>
+      </c>
+      <c r="C55" s="3">
+        <v>4400.0</v>
+      </c>
+      <c r="D55" s="9">
+        <f>IF(C54=0,"",C55/C54-1)</f>
+        <v>-0.06878306878306883</v>
+      </c>
+      <c r="E55" s="3">
+        <v>3940.0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2014/15</t>
+        </is>
+      </c>
+      <c r="B56" s="2">
+        <v>2014</v>
+      </c>
+      <c r="C56" s="3">
+        <v>5100.0</v>
+      </c>
+      <c r="D56" s="9">
+        <f>IF(C55=0,"",C56/C55-1)</f>
+        <v>0.15909090909090917</v>
+      </c>
+      <c r="E56" s="3">
+        <v>4760.0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2015/16</t>
+        </is>
+      </c>
+      <c r="B57" s="2">
+        <v>2015</v>
+      </c>
+      <c r="C57" s="3">
+        <v>5300.0</v>
+      </c>
+      <c r="D57" s="9">
+        <f>IF(C56=0,"",C57/C56-1)</f>
+        <v>0.03921568627450989</v>
+      </c>
+      <c r="E57" s="3">
+        <v>5000.0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2016/17</t>
+        </is>
+      </c>
+      <c r="B58" s="2">
+        <v>2016</v>
+      </c>
+      <c r="C58" s="3">
+        <v>7510.0</v>
+      </c>
+      <c r="D58" s="9">
+        <f>IF(C57=0,"",C58/C57-1)</f>
+        <v>0.4169811320754717</v>
+      </c>
+      <c r="E58" s="3">
+        <v>7175.0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2017/18</t>
+        </is>
+      </c>
+      <c r="B59" s="2">
+        <v>2017</v>
+      </c>
+      <c r="C59" s="3">
+        <v>7600.0</v>
+      </c>
+      <c r="D59" s="9">
+        <f>IF(C58=0,"",C59/C58-1)</f>
+        <v>0.011984021304926706</v>
+      </c>
+      <c r="E59" s="3">
+        <v>7225.0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2018/19</t>
+        </is>
+      </c>
+      <c r="B60" s="2">
+        <v>2018</v>
+      </c>
+      <c r="C60" s="3">
+        <v>7100.0</v>
+      </c>
+      <c r="D60" s="9">
+        <f>IF(C59=0,"",C60/C59-1)</f>
+        <v>-0.06578947368421051</v>
+      </c>
+      <c r="E60" s="3">
+        <v>6910.0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2019/20</t>
+        </is>
+      </c>
+      <c r="B61" s="2">
+        <v>2019</v>
+      </c>
+      <c r="C61" s="3">
+        <v>5200.0</v>
+      </c>
+      <c r="D61" s="9">
+        <f>IF(C60=0,"",C61/C60-1)</f>
+        <v>-0.2676056338028169</v>
+      </c>
+      <c r="E61" s="3">
+        <v>4900.0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020/21</t>
+        </is>
+      </c>
+      <c r="B62" s="2">
+        <v>2020</v>
+      </c>
+      <c r="C62" s="3">
+        <v>6500.0</v>
+      </c>
+      <c r="D62" s="9">
+        <f>IF(C61=0,"",C62/C61-1)</f>
+        <v>0.25</v>
+      </c>
+      <c r="E62" s="3">
+        <v>6010.0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2021/22</t>
+        </is>
+      </c>
+      <c r="B63" s="2">
+        <v>2021</v>
+      </c>
+      <c r="C63" s="3">
+        <v>4800.0</v>
+      </c>
+      <c r="D63" s="9">
+        <f>IF(C62=0,"",C63/C62-1)</f>
+        <v>-0.2615384615384615</v>
+      </c>
+      <c r="E63" s="3">
+        <v>4650.0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2022/23</t>
+        </is>
+      </c>
+      <c r="B64" s="2">
+        <v>2022</v>
+      </c>
+      <c r="C64" s="3">
+        <v>5700.0</v>
+      </c>
+      <c r="D64" s="9">
+        <f>IF(C63=0,"",C64/C63-1)</f>
+        <v>0.1875</v>
+      </c>
+      <c r="E64" s="3">
+        <v>5310.0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023/24</t>
+        </is>
+      </c>
+      <c r="B65" s="2">
+        <v>2023</v>
+      </c>
+      <c r="C65" s="3">
+        <v>5050.0</v>
+      </c>
+      <c r="D65" s="9">
+        <f>IF(C64=0,"",C65/C64-1)</f>
+        <v>-0.11403508771929827</v>
+      </c>
+      <c r="E65" s="3">
+        <v>4715.0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024/25</t>
+        </is>
+      </c>
+      <c r="B66" s="2">
+        <v>2024</v>
+      </c>
+      <c r="C66" s="3">
+        <v>5200.0</v>
+      </c>
+      <c r="D66" s="9">
+        <f>IF(C65=0,"",C66/C65-1)</f>
+        <v>0.02970297029702973</v>
+      </c>
+      <c r="E66" s="3">
+        <v>4958.0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025/26</t>
+        </is>
+      </c>
+      <c r="B67" s="2">
+        <v>2025</v>
+      </c>
+      <c r="C67" s="3">
+        <v>5530.0</v>
+      </c>
+      <c r="D67" s="9">
+        <f>IF(C66=0,"",C67/C66-1)</f>
+        <v>0.06346153846153846</v>
+      </c>
+      <c r="E67" s="3">
+        <v>5028.0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026/27</t>
+        </is>
+      </c>
+      <c r="B68" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C68" s="3">
+        <v>6030.0</v>
+      </c>
+      <c r="D68" s="9">
+        <f>IF(C67=0,"",C68/C67-1)</f>
+        <v>0.0904159132007234</v>
+      </c>
+      <c r="E68" s="3">
+        <v>5500.0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USDA PSD online, Coffee, Green, Honduras, 1000 60-kg bags, marketing year Oct-Sep, download of July 2026. 2025/26 and 2026/27 are USDA estimates and forecasts.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Varieties sheet to the Honduras area-drivers workbook
Year-by-year rust-resistant share (surveys 2013, 2014, 2017, 2020, each marked
read or unverified), Lempira share, events (releases, resistance loss, new
strains, renovation programmes), the IHCAFE releases, and an editable estimate
of the share still resistant after Lempira broke in April 2017. The deck and
the finance workbook pick up the new adoption points.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GCSUFXh2mYdWNgg7VCeE1G
</commit_message>
<xml_diff>
--- a/research/honduras/excel/Honduras_area_drivers.xlsx
+++ b/research/honduras/excel/Honduras_area_drivers.xlsx
@@ -11,7 +11,8 @@
     <sheet name="Margin" sheetId="4" r:id="rId4"/>
     <sheet name="Rust_2012" sheetId="5" r:id="rId5"/>
     <sheet name="USDA_quotes" sheetId="6" r:id="rId6"/>
-    <sheet name="Production_1960_2026" sheetId="7" r:id="rId7"/>
+    <sheet name="Varieties" sheetId="7" r:id="rId7"/>
+    <sheet name="Production_1960_2026" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,15 +20,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
     <numFmt numFmtId="167" formatCode="+#,##0;-#,##0;0"/>
     <numFmt numFmtId="168" formatCode="+0.0%;-0.0%;0.0%"/>
     <numFmt numFmtId="169" formatCode="0"/>
+    <numFmt numFmtId="170" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -81,6 +83,12 @@
     <font>
       <b/>
       <sz val="10"/>
+      <color rgb="FF2E7D32"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <color rgb="FFC00000"/>
       <name val="Arial"/>
     </font>
@@ -126,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" vertical="top"/>
@@ -152,7 +160,10 @@
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1" vertical="top"/>
     </xf>
   </cellXfs>
@@ -233,35 +244,42 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Varieties : variétés résistantes à la rouille (IHCAFE 90, Lempira, Parainema, sorties 2024), part du parc en variétés résistantes (enquêtes 2013, 2014, 2017, 2020), événements année par année, et estimation de la part encore réellement résistante après la perte de résistance de Lempira (avril 2017).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">À SAVOIR AVANT D'INTERPRÉTER</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Les nombres d'arbres de l'USDA sont des estimations : 1 049 millions chaque année de 2006 à 2010, puis une densité fixe d'environ 4 250 arbres/ha jusqu'en 2017, et 6 400/ha depuis 2023. Depuis 2020, les deux tiers de la hausse des arbres viennent de cette densité, pas de nouvelles surfaces.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">La FAO marque la surface de café du Honduras comme imputée depuis 2013 et le prix producteur comme estimé : non utilisés.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La FAO marque la surface de café du Honduras comme imputée depuis 2013 et le prix producteur comme estimé : non utilisés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Le registre de l'IHCAFE (surface récoltée des fermes inscrites) baisse de 315 700 ha (2022/23) à 280 100 (2023/24) puis 285 600 ha (2024/25), alors que l'USDA l'augmente : la hausse récente de la surface est incertaine.</t>
         </is>
@@ -5920,6 +5938,946 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
+    <col min="1" max="1" width="64" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="45" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="60" customWidth="1"/>
+    <col min="9" max="9" width="45" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rust-resistant varieties: what is planted, what still resists (2005–2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One row per marketing year. Areas come from the Annual sheet (formulas). Resistant share = only the survey figures found, never interpolated. ✔ = read in a USDA report; ⚠ = web-search extract, page blocked here, to be checked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Year (MY start)</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bearing area (1000 ha)</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non-bearing area (1000 ha)</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistant share (%)</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What the % measures</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lempira share (%)</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Event that year</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>2005</v>
+      </c>
+      <c r="B5" s="4">
+        <f>Annual!C2</f>
+        <v>184</v>
+      </c>
+      <c r="C5" s="4">
+        <f>Annual!D2</f>
+        <v>64</v>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>2006</v>
+      </c>
+      <c r="B6" s="4">
+        <f>Annual!C3</f>
+        <v>230</v>
+      </c>
+      <c r="C6" s="4">
+        <f>Annual!D3</f>
+        <v>13</v>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>2007</v>
+      </c>
+      <c r="B7" s="4">
+        <f>Annual!C4</f>
+        <v>230</v>
+      </c>
+      <c r="C7" s="4">
+        <f>Annual!D4</f>
+        <v>13</v>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>2008</v>
+      </c>
+      <c r="B8" s="4">
+        <f>Annual!C5</f>
+        <v>224</v>
+      </c>
+      <c r="C8" s="4">
+        <f>Annual!D5</f>
+        <v>20</v>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <v>2009</v>
+      </c>
+      <c r="B9" s="4">
+        <f>Annual!C6</f>
+        <v>224</v>
+      </c>
+      <c r="C9" s="4">
+        <f>Annual!D6</f>
+        <v>20</v>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2">
+        <v>2010</v>
+      </c>
+      <c r="B10" s="4">
+        <f>Annual!C7</f>
+        <v>238</v>
+      </c>
+      <c r="C10" s="4">
+        <f>Annual!D7</f>
+        <v>28</v>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2">
+        <v>2011</v>
+      </c>
+      <c r="B11" s="4">
+        <f>Annual!C8</f>
+        <v>245</v>
+      </c>
+      <c r="C11" s="4">
+        <f>Annual!D8</f>
+        <v>40</v>
+      </c>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2">
+        <v>2012</v>
+      </c>
+      <c r="B12" s="4">
+        <f>Annual!C9</f>
+        <v>267</v>
+      </c>
+      <c r="C12" s="4">
+        <f>Annual!D9</f>
+        <v>48</v>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rust epidemic starts (Central America)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2">
+        <v>2013</v>
+      </c>
+      <c r="B13" s="4">
+        <f>Annual!C10</f>
+        <v>213</v>
+      </c>
+      <c r="C13" s="4">
+        <f>Annual!D10</f>
+        <v>50</v>
+      </c>
+      <c r="D13" s="3">
+        <v>50</v>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun 2013: 50 % of national, % of coffee AREA; 2013: 50 % of national, manzanas</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">✔ USDA report (read)</t>
+        </is>
+      </c>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rust: 25 % of area hit (71 000 ha); emergency credit; 50 % of area still susceptible</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAIN 2013; El Heraldo 2013 (search snippet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2">
+        <v>2014</v>
+      </c>
+      <c r="B14" s="4">
+        <f>Annual!C11</f>
+        <v>227</v>
+      </c>
+      <c r="C14" s="4">
+        <f>Annual!D11</f>
+        <v>66</v>
+      </c>
+      <c r="D14" s="3">
+        <v>60</v>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Apr 2014: 60 % of national, % of PRODUCERS; 2014: 62 % of 5 departments (60 % of area), % of FARMS</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">✔ USDA report (read)</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">April survey: national incidence 12 %; early-warning system (SAT) set up</t>
+        </is>
+      </c>
+      <c r="I14" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAIN 2014; GAIN 2014 (USDA/TechnoServe baseline)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2">
+        <v>2015</v>
+      </c>
+      <c r="B15" s="4">
+        <f>Annual!C12</f>
+        <v>240</v>
+      </c>
+      <c r="C15" s="4">
+        <f>Annual!D12</f>
+        <v>63</v>
+      </c>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PAPP / PEPP replanting for ~23 000 small producers (1 manzana, no interest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2">
+        <v>2016</v>
+      </c>
+      <c r="B16" s="4">
+        <f>Annual!C13</f>
+        <v>280</v>
+      </c>
+      <c r="C16" s="4">
+        <f>Annual!D13</f>
+        <v>54</v>
+      </c>
+      <c r="H16" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Renovated plots start bearing</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2">
+        <v>2017</v>
+      </c>
+      <c r="B17" s="4">
+        <f>Annual!C14</f>
+        <v>298</v>
+      </c>
+      <c r="C17" s="4">
+        <f>Annual!D14</f>
+        <v>44</v>
+      </c>
+      <c r="D17" s="3">
+        <v>60</v>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aug 2017: 60 % of national coffee park (plants)</t>
+        </is>
+      </c>
+      <c r="F17" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⚠ web extract, not verified</t>
+        </is>
+      </c>
+      <c r="G17" s="6">
+        <v>56.08</v>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">April: IHCAFE confirms Lempira has lost its resistance (3 % of Lempira plants infected)</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La Prensa, 25 Aug 2017 (search extract)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2">
+        <v>2018</v>
+      </c>
+      <c r="B18" s="4">
+        <f>Annual!C15</f>
+        <v>286</v>
+      </c>
+      <c r="C18" s="4">
+        <f>Annual!D15</f>
+        <v>36</v>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">April: 4 new rust strains; Parainema and IHCAFE 90 still resistant</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2">
+        <v>2019</v>
+      </c>
+      <c r="B19" s="4">
+        <f>Annual!C16</f>
+        <v>270</v>
+      </c>
+      <c r="C19" s="4">
+        <f>Annual!D16</f>
+        <v>35</v>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">April: 16 new rust strains identified</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2">
+        <v>2020</v>
+      </c>
+      <c r="B20" s="4">
+        <f>Annual!C17</f>
+        <v>273</v>
+      </c>
+      <c r="C20" s="4">
+        <f>Annual!D17</f>
+        <v>34</v>
+      </c>
+      <c r="D20" s="3">
+        <v>60</v>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">~2020: 60 % of national, % of cultivation</t>
+        </is>
+      </c>
+      <c r="F20" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⚠ web extract, not verified</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USDA: only Parainema named as still resistant</t>
+        </is>
+      </c>
+      <c r="I20" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perfect Daily Grind, Mar 2020 (search extract)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2">
+        <v>2021</v>
+      </c>
+      <c r="B21" s="4">
+        <f>Annual!C18</f>
+        <v>275</v>
+      </c>
+      <c r="C21" s="4">
+        <f>Annual!D18</f>
+        <v>32</v>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eta and Iota: 15–25 % incidence in 5 departments (end 2020)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2">
+        <v>2022</v>
+      </c>
+      <c r="B22" s="4">
+        <f>Annual!C19</f>
+        <v>285</v>
+      </c>
+      <c r="C22" s="4">
+        <f>Annual!D19</f>
+        <v>35</v>
+      </c>
+      <c r="H22" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2">
+        <v>2023</v>
+      </c>
+      <c r="B23" s="4">
+        <f>Annual!C20</f>
+        <v>292</v>
+      </c>
+      <c r="C23" s="4">
+        <f>Annual!D20</f>
+        <v>38</v>
+      </c>
+      <c r="H23" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IHCAFE renovation programme 2023–2027: 33 000 producers, 250 000 manzanas (63 % of the park)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2">
+        <v>2024</v>
+      </c>
+      <c r="B24" s="4">
+        <f>Annual!C21</f>
+        <v>300</v>
+      </c>
+      <c r="C24" s="4">
+        <f>Annual!D21</f>
+        <v>40</v>
+      </c>
+      <c r="H24" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feb: 3 new varieties (Ihcatú 75, Anacafé 14 SHN, Obatá SHN) ⚠; seed for ≥ 1 500 manzanas</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B25" s="4">
+        <f>Annual!C22</f>
+        <v>310</v>
+      </c>
+      <c r="C25" s="4">
+        <f>Annual!D22</f>
+        <v>40</v>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USDA: area growth "driven by the introduction of the Parainema variety"; ≥ 4 more varieties announced ⚠</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B26" s="4">
+        <f>Annual!C23</f>
+        <v>330</v>
+      </c>
+      <c r="C26" s="4">
+        <f>Annual!D23</f>
+        <v>30</v>
+      </c>
+      <c r="H26" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">March: national incidence 8.44 %, highest reported since 2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Varieties released by IHCAFE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Variety</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Family</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Released</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistance status</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Release year status</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Year resistance lost</t>
+        </is>
+      </c>
+      <c r="H29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IHCAFE 90</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Catimor (Caturra × Timor Hybrid)</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1990s</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Still resistant in April 2018 (IHCAFE, 4 new rust strains found); not listed as resistant in USDA 2020 (16 new strains, April 2019)</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⚠ web extract, not verified</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H30" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAIN 2013 ("The varieties developed were the IHCAFE 90 and Lempira"); GAIN 2018; GAIN 2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lempira</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Catimor (Timor Hybrid 832/1 × Caturra)</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1997–98</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistance loss confirmed by IHCAFE in April 2017; rust on 3 % of Lempira plants</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⚠ web extract, not verified</t>
+        </is>
+      </c>
+      <c r="G31" s="14">
+        <v>2017</v>
+      </c>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAIN 2017 ("In April 2017, IHCAFE confirmed the loss of resistance of the Lempira variety"; "rust was present on three percent of Lempira variety plants")</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parainema</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sarchimor T-5296 (Villa Sarchí × Timor Hybrid)</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2004</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Still resistant per IHCAFE (USDA 2018, 2020, 2021); USDA 2025–26: area growth "driven by the introduction of the Parainema variety"</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⚠ web extract, not verified</t>
+        </is>
+      </c>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H32" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAIN 2014 (third IHCAFE variety listed); GAIN 2018; GAIN 2020; GAIN 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ihcatú 75, Anacafé 14 SHN, Obatá SHN</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 varieties presented by IHCAFE</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feb 2024</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Presented as rust resistant, productive; seed for at least 1 500 manzanas in 2024</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⚠ web extract, not verified</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H33" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El Heraldo, "Honduras dispone de tres nuevas variedades de café" (2024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 more in the pipeline</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IHCAFE research centres</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">announced</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"at least 4 more rust-resistant varieties" being prepared</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⚠ web extract, not verified</t>
+        </is>
+      </c>
+      <c r="G34" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H34" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La Prensa, "Ihcafé se prepara para liberar 4 variedades más resistentes a roya"</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After April 2017: how much of the park still resists? (order of magnitude, from two web extracts; edit the blue cells)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Share of the park in "resistant" varieties, Aug 2017 (La Prensa ⚠)</t>
+        </is>
+      </c>
+      <c r="B37" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lempira share of the farms monitored by the early-warning system, Oct 2017 (IHCAFE bulletin No 8 ⚠)</t>
+        </is>
+      </c>
+      <c r="B38" s="6">
+        <v>56.08</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Other resistant varieties (IHCAFE 90, Parainema): difference</t>
+        </is>
+      </c>
+      <c r="B39" s="5">
+        <f>MAX(0,B37-B38)</f>
+        <v>3.9200000000000017</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistance of IHCAFE 90 to the new strain, % (IHCAFE via La Prensa ⚠)</t>
+        </is>
+      </c>
+      <c r="B40" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistance of Parainema to the new strain, % (same source ⚠)</t>
+        </is>
+      </c>
+      <c r="B41" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Share of the park still resistant after April 2017, low (all IHCAFE 90)</t>
+        </is>
+      </c>
+      <c r="B42" s="5">
+        <f>B39*B40/100</f>
+        <v>3.1360000000000015</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Share of the park still resistant after April 2017, high (all Parainema)</t>
+        </is>
+      </c>
+      <c r="B43" s="5">
+        <f>B39*B41/100</f>
+        <v>3.9200000000000017</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seed demand 2017: Lempira, % (La Prensa ⚠)</t>
+        </is>
+      </c>
+      <c r="B44" s="3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seed demand 2017: other varieties (not Catuaí), %</t>
+        </is>
+      </c>
+      <c r="B45" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lempira share of resistant seed sold in 2017, at least</t>
+        </is>
+      </c>
+      <c r="B46" s="21">
+        <f>B44/(B44+B45)</f>
+        <v>0.8666666666666667</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reading: in 2013–2020 about 60 % of the park was planted with varieties called resistant, but most of it was Lempira. When Lempira broke in April 2017, the share that still resisted fell to a few percent (IHCAFE 90 and Parainema), which is why the 2023–2027 renovation targets 63 % of the park.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Caution: the two main inputs come from different samples (whole park vs farms monitored for rust) and could not be opened here. Treat the result as an order of magnitude.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not found anywhere we could reach: a yearly series of area by variety. IHCAFE publishes it in its statistical reports and coffee census (ihcafe.hn, blocked by the network policy).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="13.2"/>
+  <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>

</xml_diff>

<commit_message>
Correct the Honduras variety facts and the post-2017 resistant-share estimate
The share of monitored farms still holding a resistant variety after Lempira
failed is about 17 % (IHCAFE bulletin No 8 alone: 56.08 / 67.74), not 3-4 %
(which mixed two different samples). Parainema is shown as resistant only up
to the last explicit statement (May 2021), IHCAFE 90 as partial from 2017,
Lempira as weakening from 2015. The 2024 varieties are marked as bred abroad,
and the 4 announced varieties are replaced by the 2 in release process in 2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GCSUFXh2mYdWNgg7VCeE1G
</commit_message>
<xml_diff>
--- a/research/honduras/excel/Honduras_area_drivers.xlsx
+++ b/research/honduras/excel/Honduras_area_drivers.xlsx
@@ -6240,7 +6240,7 @@
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAPP / PEPP replanting for ~23 000 small producers (1 manzana, no interest)</t>
+          <t xml:space="preserve">PAPP / PEPP replanting for ~23 000 small producers (1 manzana, no interest); Lempira resistance weakening in IHCAFE monitoring ⚠</t>
         </is>
       </c>
     </row>
@@ -6279,7 +6279,7 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aug 2017: 60 % of national coffee park (plants)</t>
+          <t xml:space="preserve">Aug 2017: 60 % of national coffee park (plants); Oct 2017: 17 % of farms sampled by the rust early-warning system</t>
         </is>
       </c>
       <c r="F17" s="20" t="inlineStr">
@@ -6297,7 +6297,7 @@
       </c>
       <c r="I17" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">La Prensa, 25 Aug 2017 (search extract)</t>
+          <t xml:space="preserve">La Prensa, 25 Aug 2017 (search extract); IHCAFE SAT bulletin No 8 (search snippet)</t>
         </is>
       </c>
     </row>
@@ -6364,7 +6364,7 @@
       </c>
       <c r="H20" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">USDA: only Parainema named as still resistant</t>
+          <t xml:space="preserve">USDA 2020 and 2021: only Parainema named as still resistant (last explicit statement May 2021)</t>
         </is>
       </c>
       <c r="I20" s="14" t="inlineStr">
@@ -6459,7 +6459,7 @@
       </c>
       <c r="H25" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">USDA: area growth "driven by the introduction of the Parainema variety"; ≥ 4 more varieties announced ⚠</t>
+          <t xml:space="preserve">USDA: area growth "driven by the introduction of the Parainema variety"</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="H26" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">March: national incidence 8.44 %, highest reported since 2014</t>
+          <t xml:space="preserve">March: national incidence 8.44 %, highest reported since 2014; 2 more varieties in release process ⚠</t>
         </is>
       </c>
     </row>
@@ -6553,7 +6553,7 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Still resistant in April 2018 (IHCAFE, 4 new rust strains found); not listed as resistant in USDA 2020 (16 new strains, April 2019)</t>
+          <t xml:space="preserve">Still resistant per IHCAFE in April 2018 (USDA). About 80 % resistance to the new strain (IHCAFE via La Prensa, Aug 2017 ⚠). Not named as resistant by USDA after 2018</t>
         </is>
       </c>
       <c r="F30" s="14" t="inlineStr">
@@ -6568,7 +6568,7 @@
       </c>
       <c r="H30" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAIN 2013 ("The varieties developed were the IHCAFE 90 and Lempira"); GAIN 2018; GAIN 2020</t>
+          <t xml:space="preserve">GAIN 2013 ("The varieties developed were the IHCAFE 90 and Lempira"); GAIN 2018; La Prensa 2017 (extract)</t>
         </is>
       </c>
     </row>
@@ -6595,7 +6595,7 @@
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistance loss confirmed by IHCAFE in April 2017; rust on 3 % of Lempira plants</t>
+          <t xml:space="preserve">Weakening seen in IHCAFE monitoring from 2007, susceptible by 2015 (PROMECAFE 2019 ⚠); loss confirmed by IHCAFE in April 2017, rust on 3 % of Lempira plants (USDA)</t>
         </is>
       </c>
       <c r="F31" s="14" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="H31" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAIN 2017 ("In April 2017, IHCAFE confirmed the loss of resistance of the Lempira variety"; "rust was present on three percent of Lempira variety plants")</t>
+          <t xml:space="preserve">GAIN 2017 ("In April 2017, IHCAFE confirmed the loss of resistance of the Lempira variety"); PROMECAFE 24th symposium 2019 (extract)</t>
         </is>
       </c>
     </row>
@@ -6635,7 +6635,7 @@
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Still resistant per IHCAFE (USDA 2018, 2020, 2021); USDA 2025–26: area growth "driven by the introduction of the Parainema variety"</t>
+          <t xml:space="preserve">Called still resistant by IHCAFE in USDA 2018, 2020 and 2021 (last explicit statement: May 2021). Web extracts (⚠): new rust races overcome it in some zones (2019). USDA 2025–26: harvest and area growth from Parainema</t>
         </is>
       </c>
       <c r="F32" s="14" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="H32" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAIN 2014 (third IHCAFE variety listed); GAIN 2018; GAIN 2020; GAIN 2025</t>
+          <t xml:space="preserve">GAIN 2014 (third IHCAFE variety listed); GAIN 2018, 2020, 2021, 2025, 2026</t>
         </is>
       </c>
     </row>
@@ -6662,12 +6662,12 @@
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 varieties presented by IHCAFE</t>
+          <t xml:space="preserve">bred in Brazil (Icatu, Obatá) and Guatemala (Anacafé 14); validated and released by IHCAFE</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Feb 2024</t>
+          <t xml:space="preserve">2024</t>
         </is>
       </c>
       <c r="D33" s="14" t="inlineStr">
@@ -6677,7 +6677,7 @@
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Presented as rust resistant, productive; seed for at least 1 500 manzanas in 2024</t>
+          <t xml:space="preserve">Presented as rust resistant and productive; seed for at least 1 500 manzanas in 2024</t>
         </is>
       </c>
       <c r="F33" s="14" t="inlineStr">
@@ -6699,7 +6699,7 @@
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 more in the pipeline</t>
+          <t xml:space="preserve">2 more in release process</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
@@ -6709,7 +6709,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">announced</t>
+          <t xml:space="preserve">2026 (announced)</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -6719,7 +6719,7 @@
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">"at least 4 more rust-resistant varieties" being prepared</t>
+          <t xml:space="preserve">"two new varieties in the process of release: rust resistant, drought tolerant, high cup quality"</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
@@ -6734,139 +6734,156 @@
       </c>
       <c r="H34" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">La Prensa, "Ihcafé se prepara para liberar 4 variedades más resistentes a roya"</t>
+          <t xml:space="preserve">web extract, early 2026 (page not identified with certainty); an earlier La Prensa article announced 4, probably including the three of 2024</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">After April 2017: how much of the park still resists? (order of magnitude, from two web extracts; edit the blue cells)</t>
+          <t xml:space="preserve">After April 2017: how many farms still had a resistant variety? (one source: IHCAFE early-warning bulletin No 8, Oct 2017, web extract ⚠; edit the blue cells)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Share of the park in "resistant" varieties, Aug 2017 (La Prensa ⚠)</t>
-        </is>
-      </c>
-      <c r="B37" s="3">
-        <v>60</v>
+          <t xml:space="preserve">Lempira, % of all monitored farms</t>
+        </is>
+      </c>
+      <c r="B37" s="6">
+        <v>56.08</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lempira share of the farms monitored by the early-warning system, Oct 2017 (IHCAFE bulletin No 8 ⚠)</t>
+          <t xml:space="preserve">Lempira, % of the monitored farms classed as "susceptible varieties" (Lempira counted as susceptible after April 2017)</t>
         </is>
       </c>
       <c r="B38" s="6">
-        <v>56.08</v>
+        <v>67.74</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other resistant varieties (IHCAFE 90, Parainema): difference</t>
+          <t xml:space="preserve">Farms with susceptible varieties, % of all monitored farms</t>
         </is>
       </c>
       <c r="B39" s="5">
-        <f>MAX(0,B37-B38)</f>
-        <v>3.9200000000000017</v>
+        <f>B37/B38*100</f>
+        <v>82.7871272512548</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistance of IHCAFE 90 to the new strain, % (IHCAFE via La Prensa ⚠)</t>
-        </is>
-      </c>
-      <c r="B40" s="3">
-        <v>80</v>
+          <t xml:space="preserve">Farms still with a resistant variety (IHCAFE 90, Parainema, others), %</t>
+        </is>
+      </c>
+      <c r="B40" s="5">
+        <f>100-B39</f>
+        <v>17.2128727487452</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistance of Parainema to the new strain, % (same source ⚠)</t>
-        </is>
-      </c>
-      <c r="B41" s="3">
-        <v>100</v>
+          <t xml:space="preserve">Same farms before Lempira failed (Lempira + other resistant), %</t>
+        </is>
+      </c>
+      <c r="B41" s="5">
+        <f>B37+B40</f>
+        <v>73.29287274874518</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Share of the park still resistant after April 2017, low (all IHCAFE 90)</t>
-        </is>
-      </c>
-      <c r="B42" s="5">
-        <f>B39*B40/100</f>
-        <v>3.1360000000000015</v>
+          <t xml:space="preserve">For comparison: share of the whole park in "resistant" varieties, Aug 2017 (La Prensa ⚠)</t>
+        </is>
+      </c>
+      <c r="B42" s="3">
+        <v>60</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Share of the park still resistant after April 2017, high (all Parainema)</t>
-        </is>
-      </c>
-      <c r="B43" s="5">
-        <f>B39*B41/100</f>
-        <v>3.9200000000000017</v>
+          <t xml:space="preserve">Resistance of IHCAFE 90 to the new strain, % (IHCAFE via La Prensa, Aug 2017 ⚠)</t>
+        </is>
+      </c>
+      <c r="B43" s="3">
+        <v>80</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Seed demand 2017: Lempira, % (La Prensa ⚠)</t>
+          <t xml:space="preserve">Resistance of Parainema to the new strain, % (same source ⚠)</t>
         </is>
       </c>
       <c r="B44" s="3">
-        <v>65</v>
+        <v>100</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Seed demand 2017: other varieties (not Catuaí), %</t>
+          <t xml:space="preserve">Seed demand 2017: Lempira, % (La Prensa ⚠)</t>
         </is>
       </c>
       <c r="B45" s="3">
-        <v>10</v>
+        <v>65</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lempira share of resistant seed sold in 2017, at least</t>
-        </is>
-      </c>
-      <c r="B46" s="21">
-        <f>B44/(B44+B45)</f>
+          <t xml:space="preserve">Seed demand 2017: other varieties (not Catuaí), %</t>
+        </is>
+      </c>
+      <c r="B46" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lempira share of the resistant seed sold in 2017, at least</t>
+        </is>
+      </c>
+      <c r="B47" s="21">
+        <f>B45/(B45+B46)</f>
         <v>0.8666666666666667</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reading: in 2013–2020 about 60 % of the park was planted with varieties called resistant, but most of it was Lempira. When Lempira broke in April 2017, the share that still resisted fell to a few percent (IHCAFE 90 and Parainema), which is why the 2023–2027 renovation targets 63 % of the park.</t>
-        </is>
-      </c>
-    </row>
     <row r="49">
-      <c r="A49" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Caution: the two main inputs come from different samples (whole park vs farms monitored for rust) and could not be opened here. Treat the result as an order of magnitude.</t>
+      <c r="A49" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reading: in the farms IHCAFE monitored, about 73 % had a variety sold as resistant before 2017, but 56 points of it were Lempira. When Lempira failed, about 17 % were left with a variety that still resisted (IHCAFE 90 partly, Parainema). This is why the 2023–2027 renovation targets 63 % of the park.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not found anywhere we could reach: a yearly series of area by variety. IHCAFE publishes it in its statistical reports and coffee census (ihcafe.hn, blocked by the network policy).</t>
+      <c r="A50" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Correction: an earlier version of this sheet gave "3–4 %" by subtracting the bulletin figure (56 %) from the park figure (60 %). Those two numbers come from different samples; the 17 % above uses the bulletin alone and is the consistent figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Caution: the bulletin covers farms monitored for rust, not the whole park, and could not be opened here (ihcafe.hn is blocked by the network policy). Order of magnitude only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not found anywhere we could reach: a yearly series of area by variety. IHCAFE keeps it in its farm registry and statistical reports (ihcafe.hn).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Check the variety and financing slides against downloaded sources
Release years (IHCAFE 90 1990, Lempira 1998, Parainema 2004), the 65 % share
of the area in resistant varieties since 2012 and each variety's resistance
history now come from the IHCAFE study presented at the 2019 PROMECAFE
symposium, World Coffee Research pages and dated press articles. Lempira is
tolerant from 2002 and susceptible from 2016; IHCAFE 90 is 20 % susceptible
from 2016. The 2024 varieties were bred abroad; the 4 announced in Sep 2023
became the 3 released in Feb 2024. Decree 93-2018 lends L200 per quintal (not
US$25) and the BANHPROVI fund dates from 2018. The 2013 rust credit: L1,715 M
made available at 10 %, only L335 M used by April 2014.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GCSUFXh2mYdWNgg7VCeE1G
</commit_message>
<xml_diff>
--- a/research/honduras/excel/Honduras_area_drivers.xlsx
+++ b/research/honduras/excel/Honduras_area_drivers.xlsx
@@ -6060,7 +6060,7 @@
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Rust already on all Lempira plants in IHCAFE seed plots (low severity): resistance weakening (IHCAFE 2019)</t>
         </is>
       </c>
     </row>
@@ -6148,9 +6148,27 @@
         <f>Annual!D9</f>
         <v>48</v>
       </c>
+      <c r="D12" s="3">
+        <v>65</v>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">since 2012: 65 % of cultivated area, dominated by Lempira</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">✔ document read</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rust epidemic starts (Central America)</t>
+          <t xml:space="preserve">Rust epidemic starts (Central America); resistant varieties = 65 % of the area, mostly Lempira (IHCAFE 2019)</t>
+        </is>
+      </c>
+      <c r="I12" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Morales &amp; Grajeda (IHCAFE), PROMECAFE 2019 (read)</t>
         </is>
       </c>
     </row>
@@ -6171,7 +6189,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jun 2013: 50 % of national, % of coffee AREA; 2013: 50 % of national, manzanas</t>
+          <t xml:space="preserve">Jun 2013: 50 % of national, % of coffee AREA</t>
         </is>
       </c>
       <c r="F13" s="19" t="inlineStr">
@@ -6186,7 +6204,7 @@
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAIN 2013; El Heraldo 2013 (search snippet)</t>
+          <t xml:space="preserve">GAIN 2013</t>
         </is>
       </c>
     </row>
@@ -6240,7 +6258,7 @@
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAPP / PEPP replanting for ~23 000 small producers (1 manzana, no interest); Lempira resistance weakening in IHCAFE monitoring ⚠</t>
+          <t xml:space="preserve">PAPP / PEPP replanting for ~23 000 small producers (1 manzana, no interest); March: Lempira mother plants 100 % infected (IHCAFE)</t>
         </is>
       </c>
     </row>
@@ -6258,7 +6276,7 @@
       </c>
       <c r="H16" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Renovated plots start bearing</t>
+          <t xml:space="preserve">Lempira becomes susceptible (Olancho, full defoliation); ~20 % of IHCAFE 90 and Obatá plants susceptible (IHCAFE 2019); renovated plots start bearing</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6351,7 @@
       </c>
       <c r="H19" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">April: 16 new rust strains identified</t>
+          <t xml:space="preserve">April: 16 new rust strains; the Lempira-breaking rust has spread from Olancho to Copán (2017–2019); Parainema still resistant (IHCAFE)</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6441,7 @@
       </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">IHCAFE renovation programme 2023–2027: 33 000 producers, 250 000 manzanas (63 % of the park)</t>
+          <t xml:space="preserve">IHCAFE renovation programme 2023–2027: 33 000 producers, 250 000 manzanas (63 % of the park); Sep: at least 4 varieties announced for 2024</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6459,7 @@
       </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Feb: 3 new varieties (Ihcatú 75, Anacafé 14 SHN, Obatá SHN) ⚠; seed for ≥ 1 500 manzanas</t>
+          <t xml:space="preserve">29 Feb: IHCAFE presents Ihcatú 75, Anacafé 14 SHN, Obatá SHN (bred abroad; seed for ≥ 1 500 manzanas), 20 years after Parainema</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6495,7 @@
       </c>
       <c r="H26" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">March: national incidence 8.44 %, highest reported since 2014; 2 more varieties in release process ⚠</t>
+          <t xml:space="preserve">March: national incidence 8.44 %, highest reported since 2014</t>
         </is>
       </c>
     </row>
@@ -6538,12 +6556,12 @@
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Catimor (Caturra × Timor Hybrid)</t>
+          <t xml:space="preserve">Catimor (Timor Hybrid 832/1 × Caturra)</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">1990s</t>
+          <t xml:space="preserve">1990</t>
         </is>
       </c>
       <c r="D30" s="14" t="inlineStr">
@@ -6553,12 +6571,12 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Still resistant per IHCAFE in April 2018 (USDA). About 80 % resistance to the new strain (IHCAFE via La Prensa, Aug 2017 ⚠). Not named as resistant by USDA after 2018</t>
+          <t xml:space="preserve">Resistant 1990–2015; from 2016 about 20 % of plants susceptible to the new rust races (IHCAFE, 2019). USDA 2018: still resistant. World Coffee Research: "recently confirmed susceptible in Honduras"</t>
         </is>
       </c>
       <c r="F30" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">⚠ web extract, not verified</t>
+          <t xml:space="preserve">✔ document read</t>
         </is>
       </c>
       <c r="G30" s="14" t="inlineStr">
@@ -6568,7 +6586,7 @@
       </c>
       <c r="H30" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAIN 2013 ("The varieties developed were the IHCAFE 90 and Lempira"); GAIN 2018; La Prensa 2017 (extract)</t>
+          <t xml:space="preserve">Morales &amp; Grajeda (IHCAFE), PROMECAFE 24th symposium 2019, table "Durabilidad de resistencia"; GAIN 2018; WCR variety page</t>
         </is>
       </c>
     </row>
@@ -6585,7 +6603,7 @@
       </c>
       <c r="C31" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">1997–98</t>
+          <t xml:space="preserve">1998</t>
         </is>
       </c>
       <c r="D31" s="14" t="inlineStr">
@@ -6595,20 +6613,20 @@
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Weakening seen in IHCAFE monitoring from 2007, susceptible by 2015 (PROMECAFE 2019 ⚠); loss confirmed by IHCAFE in April 2017, rust on 3 % of Lempira plants (USDA)</t>
+          <t xml:space="preserve">Resistant 1998–2001; tolerant 2002–2015 (rust already on 100 % of plants, low severity, in seed plots in July 2007); susceptible in 2016 (Olancho, full defoliation), spread over the whole country 2017–2019. USDA: IHCAFE confirmed the loss in April 2017</t>
         </is>
       </c>
       <c r="F31" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">⚠ web extract, not verified</t>
+          <t xml:space="preserve">✔ document read</t>
         </is>
       </c>
       <c r="G31" s="14">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="H31" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAIN 2017 ("In April 2017, IHCAFE confirmed the loss of resistance of the Lempira variety"); PROMECAFE 24th symposium 2019 (extract)</t>
+          <t xml:space="preserve">Morales &amp; Grajeda (IHCAFE), PROMECAFE 2019; GAIN 2017; WCR variety page</t>
         </is>
       </c>
     </row>
@@ -6620,7 +6638,7 @@
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sarchimor T-5296 (Villa Sarchí × Timor Hybrid)</t>
+          <t xml:space="preserve">Sarchimor, selection of T5296</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
@@ -6635,12 +6653,12 @@
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Called still resistant by IHCAFE in USDA 2018, 2020 and 2021 (last explicit statement: May 2021). Web extracts (⚠): new rust races overcome it in some zones (2019). USDA 2025–26: harvest and area growth from Parainema</t>
+          <t xml:space="preserve">Resistant 2004–2019 in IHCAFE tests (fully resistant to the new races); USDA 2018, 2020, 2021: still resistant. Nothing later found</t>
         </is>
       </c>
       <c r="F32" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">⚠ web extract, not verified</t>
+          <t xml:space="preserve">✔ document read</t>
         </is>
       </c>
       <c r="G32" s="14" t="inlineStr">
@@ -6650,7 +6668,7 @@
       </c>
       <c r="H32" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAIN 2014 (third IHCAFE variety listed); GAIN 2018, 2020, 2021, 2025, 2026</t>
+          <t xml:space="preserve">Morales &amp; Grajeda (IHCAFE), PROMECAFE 2019; WCR ("released in 2004"); GAIN 2018, 2020, 2021, 2025</t>
         </is>
       </c>
     </row>
@@ -6662,12 +6680,12 @@
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">bred in Brazil (Icatu, Obatá) and Guatemala (Anacafé 14); validated and released by IHCAFE</t>
+          <t xml:space="preserve">bred abroad (Brazil: Icatu, Obatá by IAC; Guatemala: Anacafé 14), released by IHCAFE</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024</t>
+          <t xml:space="preserve">Feb 2024</t>
         </is>
       </c>
       <c r="D33" s="14" t="inlineStr">
@@ -6677,12 +6695,12 @@
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Presented as rust resistant and productive; seed for at least 1 500 manzanas in 2024</t>
+          <t xml:space="preserve">Presented as more rust resistant and productive; seed for at least 1 500 manzanas in 2024. Caution: IHCAFE's 2019 study listed the Icatu 75 line as susceptible since 2016 and Obatá as 20 % susceptible</t>
         </is>
       </c>
       <c r="F33" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">⚠ web extract, not verified</t>
+          <t xml:space="preserve">✔ document read</t>
         </is>
       </c>
       <c r="G33" s="14" t="inlineStr">
@@ -6692,196 +6710,154 @@
       </c>
       <c r="H33" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">El Heraldo, "Honduras dispone de tres nuevas variedades de café" (2024)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 more in release process</t>
-        </is>
-      </c>
-      <c r="B34" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IHCAFE research centres</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026 (announced)</t>
-        </is>
-      </c>
-      <c r="D34" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E34" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"two new varieties in the process of release: rust resistant, drought tolerant, high cup quality"</t>
-        </is>
-      </c>
-      <c r="F34" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">⚠ web extract, not verified</t>
-        </is>
-      </c>
-      <c r="G34" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H34" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">web extract, early 2026 (page not identified with certainty); an earlier La Prensa article announced 4, probably including the three of 2024</t>
+          <t xml:space="preserve">El Heraldo, 29 Feb 2024 (read); La Prensa, 29 Sep 2023 (read: "at least 4" to be released in 2024; last release Parainema 2004); PROMECAFE 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After April 2017: how many farms still had a resistant variety? (one source: IHCAFE early-warning bulletin No 8, Oct 2017, web extract ⚠; edit the blue cells)</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">After April 2017: how many farms still had a resistant variety? (one source: IHCAFE early-warning bulletin No 8, Oct 2017, web extract ⚠; edit the blue cells)</t>
-        </is>
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lempira, % of all monitored farms</t>
+        </is>
+      </c>
+      <c r="B36" s="6">
+        <v>56.08</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lempira, % of all monitored farms</t>
+          <t xml:space="preserve">Lempira, % of the monitored farms classed as "susceptible varieties" (Lempira counted as susceptible after April 2017)</t>
         </is>
       </c>
       <c r="B37" s="6">
-        <v>56.08</v>
+        <v>67.74</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lempira, % of the monitored farms classed as "susceptible varieties" (Lempira counted as susceptible after April 2017)</t>
-        </is>
-      </c>
-      <c r="B38" s="6">
-        <v>67.74</v>
+          <t xml:space="preserve">Farms with susceptible varieties, % of all monitored farms</t>
+        </is>
+      </c>
+      <c r="B38" s="5">
+        <f>B36/B37*100</f>
+        <v>82.7871272512548</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farms with susceptible varieties, % of all monitored farms</t>
+          <t xml:space="preserve">Farms still with a resistant variety (IHCAFE 90, Parainema, others), %</t>
         </is>
       </c>
       <c r="B39" s="5">
-        <f>B37/B38*100</f>
-        <v>82.7871272512548</v>
+        <f>100-B38</f>
+        <v>17.2128727487452</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farms still with a resistant variety (IHCAFE 90, Parainema, others), %</t>
+          <t xml:space="preserve">Same farms before Lempira failed (Lempira + other resistant), %</t>
         </is>
       </c>
       <c r="B40" s="5">
-        <f>100-B39</f>
-        <v>17.2128727487452</v>
+        <f>B36+B39</f>
+        <v>73.29287274874518</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Same farms before Lempira failed (Lempira + other resistant), %</t>
-        </is>
-      </c>
-      <c r="B41" s="5">
-        <f>B37+B40</f>
-        <v>73.29287274874518</v>
+          <t xml:space="preserve">For comparison: share of the whole park in "resistant" varieties, Aug 2017 (La Prensa ⚠)</t>
+        </is>
+      </c>
+      <c r="B41" s="3">
+        <v>60</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">For comparison: share of the whole park in "resistant" varieties, Aug 2017 (La Prensa ⚠)</t>
+          <t xml:space="preserve">Resistance of IHCAFE 90 to the new strain, % (IHCAFE via La Prensa, Aug 2017 ⚠)</t>
         </is>
       </c>
       <c r="B42" s="3">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistance of IHCAFE 90 to the new strain, % (IHCAFE via La Prensa, Aug 2017 ⚠)</t>
+          <t xml:space="preserve">Resistance of Parainema to the new strain, % (same source ⚠)</t>
         </is>
       </c>
       <c r="B43" s="3">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistance of Parainema to the new strain, % (same source ⚠)</t>
+          <t xml:space="preserve">Seed demand 2017: Lempira, % (La Prensa ⚠)</t>
         </is>
       </c>
       <c r="B44" s="3">
-        <v>100</v>
+        <v>65</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Seed demand 2017: Lempira, % (La Prensa ⚠)</t>
+          <t xml:space="preserve">Seed demand 2017: other varieties (not Catuaí), %</t>
         </is>
       </c>
       <c r="B45" s="3">
-        <v>65</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Seed demand 2017: other varieties (not Catuaí), %</t>
-        </is>
-      </c>
-      <c r="B46" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="14" t="inlineStr">
-        <is>
           <t xml:space="preserve">Lempira share of the resistant seed sold in 2017, at least</t>
         </is>
       </c>
-      <c r="B47" s="21">
-        <f>B45/(B45+B46)</f>
+      <c r="B46" s="21">
+        <f>B44/(B44+B45)</f>
         <v>0.8666666666666667</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reading: in the farms IHCAFE monitored, about 73 % had a variety sold as resistant before 2017, but 56 points of it were Lempira. When Lempira failed, about 17 % were left with a variety that still resisted (IHCAFE 90 partly, Parainema). This is why the 2023–2027 renovation targets 63 % of the park.</t>
+        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reading: in the farms IHCAFE monitored, about 73 % had a variety sold as resistant before 2017, but 56 points of it were Lempira. When Lempira failed, about 17 % were left with a variety that still resisted (IHCAFE 90 partly, Parainema). This is why the 2023–2027 renovation targets 63 % of the park.</t>
+          <t xml:space="preserve">Correction: an earlier version of this sheet gave "3–4 %" by subtracting the bulletin figure (56 %) from the park figure (60 %). Those two numbers come from different samples; the 17 % above uses the bulletin alone and is the consistent figure.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Correction: an earlier version of this sheet gave "3–4 %" by subtracting the bulletin figure (56 %) from the park figure (60 %). Those two numbers come from different samples; the 17 % above uses the bulletin alone and is the consistent figure.</t>
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Caution: the bulletin covers farms monitored for rust, not the whole park, and could not be opened here (ihcafe.hn is blocked by the network policy). Order of magnitude only.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Caution: the bulletin covers farms monitored for rust, not the whole park, and could not be opened here (ihcafe.hn is blocked by the network policy). Order of magnitude only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Not found anywhere we could reach: a yearly series of area by variety. IHCAFE keeps it in its farm registry and statistical reports (ihcafe.hn).</t>
         </is>

</xml_diff>

<commit_message>
Verify the August 2017 resistant-share figure and drop the unsourced seed-demand split
La Prensa of 24 Aug 2017 (downloaded) confirms 60 % of the national coffee
park in improved rust-resistant plants and IHCAFE 90 at 80 % / Parainema at
100 % resistance to the new strain. The 65 % Lempira seed-demand figure is not
in that article; its source could not be found, so it is removed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GCSUFXh2mYdWNgg7VCeE1G
</commit_message>
<xml_diff>
--- a/research/honduras/excel/Honduras_area_drivers.xlsx
+++ b/research/honduras/excel/Honduras_area_drivers.xlsx
@@ -20,14 +20,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
     <numFmt numFmtId="167" formatCode="+#,##0;-#,##0;0"/>
     <numFmt numFmtId="168" formatCode="+0.0%;-0.0%;0.0%"/>
     <numFmt numFmtId="169" formatCode="0"/>
-    <numFmt numFmtId="170" formatCode="0.0%"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -134,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" vertical="top"/>
@@ -162,7 +161,6 @@
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1" vertical="top"/>
     </xf>
@@ -265,7 +263,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">Les nombres d'arbres de l'USDA sont des estimations : 1 049 millions chaque année de 2006 à 2010, puis une densité fixe d'environ 4 250 arbres/ha jusqu'en 2017, et 6 400/ha depuis 2023. Depuis 2020, les deux tiers de la hausse des arbres viennent de cette densité, pas de nouvelles surfaces.</t>
         </is>
@@ -6297,12 +6295,12 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aug 2017: 60 % of national coffee park (plants); Oct 2017: 17 % of farms sampled by the rust early-warning system</t>
-        </is>
-      </c>
-      <c r="F17" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">⚠ web extract, not verified</t>
+          <t xml:space="preserve">24 Aug 2017: 60 % of national coffee park (plants); Oct 2017: 17 % of farms sampled by the rust early-warning system</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">✔ document read</t>
         </is>
       </c>
       <c r="G17" s="6">
@@ -6315,7 +6313,7 @@
       </c>
       <c r="I17" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">La Prensa, 25 Aug 2017 (search extract); IHCAFE SAT bulletin No 8 (search snippet)</t>
+          <t xml:space="preserve">La Prensa, 24 Aug 2017 (read, ihcafe_docs3); IHCAFE SAT bulletin No 8 (search snippet)</t>
         </is>
       </c>
     </row>
@@ -6571,7 +6569,7 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistant 1990–2015; from 2016 about 20 % of plants susceptible to the new rust races (IHCAFE, 2019). USDA 2018: still resistant. World Coffee Research: "recently confirmed susceptible in Honduras"</t>
+          <t xml:space="preserve">Resistant 1990–2015; from 2016 about 20 % of plants susceptible to the new rust races (IHCAFE, 2019); 80 % resistance to the new strain (IHCAFE via La Prensa, 24 Aug 2017). USDA 2018: still resistant. World Coffee Research: "recently confirmed susceptible in Honduras"</t>
         </is>
       </c>
       <c r="F30" s="14" t="inlineStr">
@@ -6777,7 +6775,7 @@
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">For comparison: share of the whole park in "resistant" varieties, Aug 2017 (La Prensa ⚠)</t>
+          <t xml:space="preserve">For comparison: share of the whole park in "resistant" varieties, 24 Aug 2017 (La Prensa, read)</t>
         </is>
       </c>
       <c r="B41" s="3">
@@ -6787,7 +6785,7 @@
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistance of IHCAFE 90 to the new strain, % (IHCAFE via La Prensa, Aug 2017 ⚠)</t>
+          <t xml:space="preserve">Resistance of IHCAFE 90 to the new strain, % (IHCAFE via La Prensa, 24 Aug 2017, read)</t>
         </is>
       </c>
       <c r="B42" s="3">
@@ -6797,67 +6795,36 @@
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistance of Parainema to the new strain, % (same source ⚠)</t>
+          <t xml:space="preserve">Resistance of Parainema to the new strain, % (same source, read)</t>
         </is>
       </c>
       <c r="B43" s="3">
         <v>100</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Seed demand 2017: Lempira, % (La Prensa ⚠)</t>
-        </is>
-      </c>
-      <c r="B44" s="3">
-        <v>65</v>
-      </c>
-    </row>
     <row r="45">
-      <c r="A45" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Seed demand 2017: other varieties (not Catuaí), %</t>
-        </is>
-      </c>
-      <c r="B45" s="3">
-        <v>10</v>
+      <c r="A45" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reading: in the farms IHCAFE monitored, about 73 % had a variety sold as resistant before 2017, but 56 points of it were Lempira. When Lempira failed, about 17 % were left with a variety that still resisted (IHCAFE 90 partly, Parainema). This is why the 2023–2027 renovation targets 63 % of the park.</t>
+        </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lempira share of the resistant seed sold in 2017, at least</t>
-        </is>
-      </c>
-      <c r="B46" s="21">
-        <f>B44/(B44+B45)</f>
-        <v>0.8666666666666667</v>
+      <c r="A46" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Correction: an earlier version of this sheet gave "3–4 %" by subtracting the bulletin figure (56 %) from the park figure (60 %). Those two numbers come from different samples; the 17 % above uses the bulletin alone and is the consistent figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Caution: the bulletin covers farms monitored for rust, not the whole park, and could not be opened here (ihcafe.hn is blocked by the network policy). Order of magnitude only.</t>
+        </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reading: in the farms IHCAFE monitored, about 73 % had a variety sold as resistant before 2017, but 56 points of it were Lempira. When Lempira failed, about 17 % were left with a variety that still resisted (IHCAFE 90 partly, Parainema). This is why the 2023–2027 renovation targets 63 % of the park.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Correction: an earlier version of this sheet gave "3–4 %" by subtracting the bulletin figure (56 %) from the park figure (60 %). Those two numbers come from different samples; the 17 % above uses the bulletin alone and is the consistent figure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Caution: the bulletin covers farms monitored for rust, not the whole park, and could not be opened here (ihcafe.hn is blocked by the network policy). Order of magnitude only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="14" t="inlineStr">
+      <c r="A48" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Not found anywhere we could reach: a yearly series of area by variety. IHCAFE keeps it in its farm registry and statistical reports (ihcafe.hn).</t>
         </is>

</xml_diff>